<commit_message>
Primer commit plataforma gestion flota
</commit_message>
<xml_diff>
--- a/reporte_viajes.xlsx
+++ b/reporte_viajes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,6 +732,37 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cartagena</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sincelejo</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BBB-100</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>180</v>
+      </c>
+      <c r="F11" t="n">
+        <v>288000</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2 h 15 min</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>